<commit_message>
Udokumentuj 6 defektów wg wytycznych (rejestr + wiersze Negatywne)
DEFEKTY.md: pełna struktura na defekt (ID, tytuł, istotność, środowisko,
szczegółowe kroki, opis słowny, rezultat oczekiwany, korelacja z testami).
3 potwierdzone wyjątkiem + 3 ograniczenia. Środowisko: Linux.
TestCases_Cien_nad_Arkham.xlsx: DEF-1..DEF-6 (Negatywne) z korelacją do testów.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REFACTOR/docs/TestCases_Cien_nad_Arkham.xlsx
+++ b/REFACTOR/docs/TestCases_Cien_nad_Arkham.xlsx
@@ -1046,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:W43"/>
+  <dimension ref="B2:W49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.85546875" customWidth="1" min="2" max="2"/>
@@ -3301,6 +3301,322 @@
       </c>
       <c r="J43" s="65" t="inlineStr"/>
       <c r="K43" s="84" t="inlineStr"/>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="B44" s="65" t="inlineStr">
+        <is>
+          <t>DEF-1</t>
+        </is>
+      </c>
+      <c r="C44" s="84" t="inlineStr">
+        <is>
+          <t>Wczytanie zapisu z nieistniejącą sceną</t>
+        </is>
+      </c>
+      <c r="D44" s="84" t="inlineStr">
+        <is>
+          <t>Test destruktywny</t>
+        </is>
+      </c>
+      <c r="E44" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 + tkinter</t>
+        </is>
+      </c>
+      <c r="F44" s="65" t="inlineStr">
+        <is>
+          <t>Krytyczny</t>
+        </is>
+      </c>
+      <c r="G44" s="84" t="inlineStr">
+        <is>
+          <t>1. W data/save.json zmień 'obecny_wezel' na nieistniejącą nazwę
+2. W menu kliknij KONTYNUUJ</t>
+        </is>
+      </c>
+      <c r="H44" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie, czy gra łagodnie obsługuje błędny zapis (komunikat / powrót do menu)</t>
+        </is>
+      </c>
+      <c r="I44" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J44" s="65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K44" s="84" t="inlineStr">
+        <is>
+          <t>Wyjątek AttributeError ('NoneType' object has no attribute 'get') w odswiez_scene; brak kontroli None po pobierz_wezel  Powiązane testy: A10, A9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="B45" s="65" t="inlineStr">
+        <is>
+          <t>DEF-2</t>
+        </is>
+      </c>
+      <c r="C45" s="84" t="inlineStr">
+        <is>
+          <t>Literówka w polu 'cel' w fabule</t>
+        </is>
+      </c>
+      <c r="D45" s="84" t="inlineStr">
+        <is>
+          <t>Test destruktywny</t>
+        </is>
+      </c>
+      <c r="E45" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 + tkinter</t>
+        </is>
+      </c>
+      <c r="F45" s="65" t="inlineStr">
+        <is>
+          <t>Wysoki</t>
+        </is>
+      </c>
+      <c r="G45" s="84" t="inlineStr">
+        <is>
+          <t>1. W story.json ustaw 'cel' wyboru na nieistniejącą scenę
+2. Kliknij ten wybór</t>
+        </is>
+      </c>
+      <c r="H45" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie bezpiecznej obsługi błędnego celu (bez przerwania gry)</t>
+        </is>
+      </c>
+      <c r="I45" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J45" s="65" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K45" s="84" t="inlineStr">
+        <is>
+          <t>Silnik wypisuje błąd, ale ustawia obecny_wezel i odswiez_scene wywala AttributeError (None)  Powiązane testy: D9, C6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="B46" s="65" t="inlineStr">
+        <is>
+          <t>DEF-3</t>
+        </is>
+      </c>
+      <c r="C46" s="84" t="inlineStr">
+        <is>
+          <t>Tryb konsolowy engine.py z katalogu projektu</t>
+        </is>
+      </c>
+      <c r="D46" s="84" t="inlineStr">
+        <is>
+          <t>Test destruktywny</t>
+        </is>
+      </c>
+      <c r="E46" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 (konsola)</t>
+        </is>
+      </c>
+      <c r="F46" s="65" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="G46" s="84" t="inlineStr">
+        <is>
+          <t>1. Z katalogu projektu uruchom: python REFACTOR/engine.py</t>
+        </is>
+      </c>
+      <c r="H46" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie, czy uruchamia się konsolowy tryb gry</t>
+        </is>
+      </c>
+      <c r="I46" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J46" s="65" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K46" s="84" t="inlineStr">
+        <is>
+          <t>FileNotFoundError - open('data/config.json') używa ścieżki względnej do cwd, nie do pliku; działa tylko z wnętrza REFACTOR  Powiązane testy: C4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="B47" s="65" t="inlineStr">
+        <is>
+          <t>DEF-4</t>
+        </is>
+      </c>
+      <c r="C47" s="84" t="inlineStr">
+        <is>
+          <t>Brak przewijania długiej sceny</t>
+        </is>
+      </c>
+      <c r="D47" s="84" t="inlineStr">
+        <is>
+          <t>Test funkcjonalności</t>
+        </is>
+      </c>
+      <c r="E47" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 + tkinter</t>
+        </is>
+      </c>
+      <c r="F47" s="65" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="G47" s="84" t="inlineStr">
+        <is>
+          <t>1. Wejdź do sceny z długim tekstem i kilkoma wyborami (małe okno 592x456)</t>
+        </is>
+      </c>
+      <c r="H47" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie, czy cała treść (wszystkie przyciski) jest dostępna</t>
+        </is>
+      </c>
+      <c r="I47" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J47" s="65" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K47" s="84" t="inlineStr">
+        <is>
+          <t>Ostatnie przyciski mogą wyjść poza otwór i schować się pod ramką; brak paska przewijania  Powiązane testy: B5, B10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="B48" s="65" t="inlineStr">
+        <is>
+          <t>DEF-5</t>
+        </is>
+      </c>
+      <c r="C48" s="84" t="inlineStr">
+        <is>
+          <t>Zmiana rozmiaru okna rozjeżdża układ</t>
+        </is>
+      </c>
+      <c r="D48" s="84" t="inlineStr">
+        <is>
+          <t>Test kompatybilności</t>
+        </is>
+      </c>
+      <c r="E48" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 + tkinter</t>
+        </is>
+      </c>
+      <c r="F48" s="65" t="inlineStr">
+        <is>
+          <t>Niski</t>
+        </is>
+      </c>
+      <c r="G48" s="84" t="inlineStr">
+        <is>
+          <t>1. Uruchom grę i zmaksymalizuj / rozciągnij okno</t>
+        </is>
+      </c>
+      <c r="H48" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie, czy układ dopasowuje się do rozmiaru okna</t>
+        </is>
+      </c>
+      <c r="I48" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J48" s="65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K48" s="84" t="inlineStr">
+        <is>
+          <t>Ramka i współrzędne liczone raz w utworz_okno; po zmianie rozmiaru pusty obszar, treść się nie skaluje  Powiązane testy: A3, A6, A7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="42" customHeight="1">
+      <c r="B49" s="65" t="inlineStr">
+        <is>
+          <t>DEF-6</t>
+        </is>
+      </c>
+      <c r="C49" s="84" t="inlineStr">
+        <is>
+          <t>Nadpisanie zapisu bez ostrzeżenia</t>
+        </is>
+      </c>
+      <c r="D49" s="84" t="inlineStr">
+        <is>
+          <t>Test funkcjonalności</t>
+        </is>
+      </c>
+      <c r="E49" s="65" t="inlineStr">
+        <is>
+          <t>Linux / Python 3 + tkinter</t>
+        </is>
+      </c>
+      <c r="F49" s="65" t="inlineStr">
+        <is>
+          <t>Niski</t>
+        </is>
+      </c>
+      <c r="G49" s="84" t="inlineStr">
+        <is>
+          <t>1. Zapisz grę
+2. Zagraj dalej
+3. Zapisz ponownie</t>
+        </is>
+      </c>
+      <c r="H49" s="84" t="inlineStr">
+        <is>
+          <t>1. Sprawdzenie, czy gra ostrzega przed nadpisaniem poprzedniego zapisu</t>
+        </is>
+      </c>
+      <c r="I49" s="65" t="inlineStr">
+        <is>
+          <t>Negatywny</t>
+        </is>
+      </c>
+      <c r="J49" s="65" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K49" s="84" t="inlineStr">
+        <is>
+          <t>zapisz_gre od razu nadpisuje save.json (jeden slot), brak potwierdzenia; poprzedni stan tracony  Powiązane testy: A10.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>